<commit_message>
Warehouse allocation and LSP verfications
</commit_message>
<xml_diff>
--- a/KBL-Business flow/target/Data/KBL datas2.xlsx
+++ b/KBL-Business flow/target/Data/KBL datas2.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="24">
   <si>
     <t>1037</t>
   </si>
@@ -58,6 +58,36 @@
   </si>
   <si>
     <t>1029</t>
+  </si>
+  <si>
+    <t>1013</t>
+  </si>
+  <si>
+    <t>1024</t>
+  </si>
+  <si>
+    <t>1019</t>
+  </si>
+  <si>
+    <t>1011</t>
+  </si>
+  <si>
+    <t>1033</t>
+  </si>
+  <si>
+    <t>1034</t>
+  </si>
+  <si>
+    <t>1005</t>
+  </si>
+  <si>
+    <t>1006</t>
+  </si>
+  <si>
+    <t>1007</t>
+  </si>
+  <si>
+    <t>1003</t>
   </si>
 </sst>
 </file>
@@ -414,144 +444,162 @@
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" t="s" s="2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" t="s" s="2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" t="s" s="2">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
       <c r="A4" t="s" s="2">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" t="s" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" t="s" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" t="s" s="2">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
       <c r="A8" t="s" s="2">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
       <c r="A9" t="s" s="2">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
       <c r="A10" t="s" s="2">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" t="s" s="2">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
       <c r="A12" t="s" s="2">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
       <c r="A13" t="s" s="2">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
       <c r="A14" t="s" s="2">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="1"/>
+      <c r="A15" t="s" s="2">
+        <v>4</v>
+      </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="1"/>
+      <c r="A16" t="s" s="2">
+        <v>17</v>
+      </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="1"/>
+      <c r="A17" t="s" s="2">
+        <v>18</v>
+      </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="1"/>
+      <c r="A18" t="s" s="2">
+        <v>19</v>
+      </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="1"/>
+      <c r="A19" t="s" s="2">
+        <v>12</v>
+      </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="1"/>
+      <c r="A20" t="s" s="2">
+        <v>20</v>
+      </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="1"/>
+      <c r="A21" t="s" s="2">
+        <v>21</v>
+      </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="1"/>
+      <c r="A22" t="s" s="2">
+        <v>22</v>
+      </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="1"/>
+      <c r="A23" t="s" s="2">
+        <v>23</v>
+      </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
     </row>

</xml_diff>